<commit_message>
Remove obsolete Tailwind CSS reference documents and web design guidelines; update filters to improve house context handling; modify retailer marking page for better house filtering and add translations for filtering; update skills-lock.json to include xlsx skill.
</commit_message>
<xml_diff>
--- a/backend/data/products.xlsx
+++ b/backend/data/products.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nabeeha\projects\Orange-Flow-Next-Js\backend\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\emil\projects\Orange-Flow-Next-Js\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA57E89-2695-4316-B326-83E370EFF54B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2560217-2C83-4DC0-AECC-CB38F0792F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="23715" windowHeight="14550" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="49">
   <si>
     <t>PRODUCT_CODE</t>
   </si>
@@ -180,6 +180,9 @@
   </si>
   <si>
     <t>SIM SWAP</t>
+  </si>
+  <si>
+    <t>Tozed T30 Plus</t>
   </si>
 </sst>
 </file>
@@ -520,19 +523,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -558,7 +561,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -581,7 +584,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -604,7 +607,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -627,7 +630,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -650,7 +653,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -673,7 +676,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -696,7 +699,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -719,7 +722,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -742,7 +745,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -768,7 +771,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -794,7 +797,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -820,7 +823,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -846,7 +849,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -872,7 +875,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -898,7 +901,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -924,7 +927,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -950,7 +953,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -976,7 +979,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -985,6 +988,9 @@
       </c>
       <c r="C19" t="s">
         <v>30</v>
+      </c>
+      <c r="D19" t="s">
+        <v>48</v>
       </c>
       <c r="E19">
         <v>3300</v>

</xml_diff>